<commit_message>
new updates to code
</commit_message>
<xml_diff>
--- a/api/data/templates/Account_Setup_and_Data_Load_PM-C_template.xlsx
+++ b/api/data/templates/Account_Setup_and_Data_Load_PM-C_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gandhi/GandhiMain/700-Apps/envizi-integration-hub/app/data/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/siraj/INDRA/integration_hub_v2/api/data/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A97A921D-2DDB-DD4D-8018-DCD4D42A6635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C6572B7-BC99-C545-8971-6F46CD82B374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="29920" windowHeight="17420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="7" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Location</t>
   </si>
@@ -83,9 +83,6 @@
     <t>Record Data Quality</t>
   </si>
   <si>
-    <t>IBM APAC</t>
-  </si>
-  <si>
     <t>Organization Link</t>
   </si>
   <si>
@@ -113,34 +110,7 @@
     <t>Total Cost</t>
   </si>
   <si>
-    <t>Actual</t>
-  </si>
-  <si>
-    <t>Standard</t>
-  </si>
-  <si>
-    <t>Default</t>
-  </si>
-  <si>
-    <t>Overwrite</t>
-  </si>
-  <si>
     <t>Quantity</t>
-  </si>
-  <si>
-    <t>IN Bank -  Frankfurt Br</t>
-  </si>
-  <si>
-    <t>No Scope - Water - gallons</t>
-  </si>
-  <si>
-    <t>IN Bank -  Frankfurt Br-Water</t>
-  </si>
-  <si>
-    <t>S1 - Ethanol E10 Transport - gal</t>
-  </si>
-  <si>
-    <t>IN Bank -  Frankfurt Br-E10</t>
   </si>
 </sst>
 </file>
@@ -461,12 +431,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A3689F4-4FC5-BF45-B5C2-2D5238BB1D41}">
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:U1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1" t="s">
         <v>6</v>
@@ -475,16 +445,16 @@
         <v>0</v>
       </c>
       <c r="D1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" t="s">
         <v>16</v>
-      </c>
-      <c r="E1" t="s">
-        <v>17</v>
       </c>
       <c r="F1" t="s">
         <v>7</v>
       </c>
       <c r="G1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H1" t="s">
         <v>1</v>
@@ -496,7 +466,7 @@
         <v>8</v>
       </c>
       <c r="K1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L1" t="s">
         <v>9</v>
@@ -508,13 +478,13 @@
         <v>13</v>
       </c>
       <c r="O1" t="s">
+        <v>19</v>
+      </c>
+      <c r="P1" t="s">
         <v>20</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>21</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>22</v>
       </c>
       <c r="R1" t="s">
         <v>11</v>
@@ -523,74 +493,10 @@
         <v>12</v>
       </c>
       <c r="T1" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="U1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>17000104</v>
-      </c>
-      <c r="B2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E2">
-        <v>14795</v>
-      </c>
-      <c r="F2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H2" t="s">
-        <v>31</v>
-      </c>
-      <c r="N2" t="s">
-        <v>24</v>
-      </c>
-      <c r="O2" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>17000104</v>
-      </c>
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3">
-        <v>14454</v>
-      </c>
-      <c r="F3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H3" t="s">
-        <v>33</v>
-      </c>
-      <c r="N3" t="s">
-        <v>24</v>
-      </c>
-      <c r="O3" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>